<commit_message>
complete code for M2 and M3
</commit_message>
<xml_diff>
--- a/data/master_flat_table.xlsx
+++ b/data/master_flat_table.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE2"/>
+  <dimension ref="A1:BF2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -547,6 +547,7 @@
     <col width="14" customWidth="1" min="55" max="55"/>
     <col width="14" customWidth="1" min="56" max="56"/>
     <col width="14" customWidth="1" min="57" max="57"/>
+    <col width="14" customWidth="1" min="58" max="58"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -574,285 +575,290 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
           <t>row_id</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>patient_name</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>gender</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>year_of_birth</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>mobile_number</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>abha_address</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>abha_number</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>eka_patient_id</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>partner_patient_id</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>hip_id</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
+      <c r="L2" s="6" t="inlineStr">
         <is>
           <t>clinic_id</t>
         </is>
       </c>
-      <c r="L2" s="6" t="inlineStr">
+      <c r="M2" s="6" t="inlineStr">
         <is>
           <t>source_event_type</t>
         </is>
       </c>
-      <c r="M2" s="6" t="inlineStr">
+      <c r="N2" s="6" t="inlineStr">
         <is>
           <t>encounter_id</t>
         </is>
       </c>
-      <c r="N2" s="6" t="inlineStr">
+      <c r="O2" s="6" t="inlineStr">
         <is>
           <t>encounter_date</t>
         </is>
       </c>
-      <c r="O2" s="6" t="inlineStr">
+      <c r="P2" s="6" t="inlineStr">
         <is>
           <t>practitioner_name</t>
         </is>
       </c>
-      <c r="P2" s="6" t="inlineStr">
+      <c r="Q2" s="6" t="inlineStr">
         <is>
           <t>symptoms_text</t>
         </is>
       </c>
-      <c r="Q2" s="6" t="inlineStr">
+      <c r="R2" s="6" t="inlineStr">
         <is>
           <t>symptoms_snomed_code</t>
         </is>
       </c>
-      <c r="R2" s="6" t="inlineStr">
+      <c r="S2" s="6" t="inlineStr">
         <is>
           <t>vitals_bp_systolic</t>
         </is>
       </c>
-      <c r="S2" s="6" t="inlineStr">
+      <c r="T2" s="6" t="inlineStr">
         <is>
           <t>vitals_bp_diastolic</t>
         </is>
       </c>
-      <c r="T2" s="6" t="inlineStr">
+      <c r="U2" s="6" t="inlineStr">
         <is>
           <t>vitals_pulse</t>
         </is>
       </c>
-      <c r="U2" s="6" t="inlineStr">
+      <c r="V2" s="6" t="inlineStr">
         <is>
           <t>vitals_temp_c</t>
         </is>
       </c>
-      <c r="V2" s="6" t="inlineStr">
+      <c r="W2" s="6" t="inlineStr">
         <is>
           <t>vitals_spo2</t>
         </is>
       </c>
-      <c r="W2" s="6" t="inlineStr">
+      <c r="X2" s="6" t="inlineStr">
         <is>
           <t>examination_notes</t>
         </is>
       </c>
-      <c r="X2" s="6" t="inlineStr">
+      <c r="Y2" s="6" t="inlineStr">
         <is>
           <t>diagnosis_text</t>
         </is>
       </c>
-      <c r="Y2" s="6" t="inlineStr">
+      <c r="Z2" s="6" t="inlineStr">
         <is>
           <t>diagnosis_snomed_code</t>
         </is>
       </c>
-      <c r="Z2" s="6" t="inlineStr">
+      <c r="AA2" s="6" t="inlineStr">
         <is>
           <t>medical_history_text</t>
         </is>
       </c>
-      <c r="AA2" s="6" t="inlineStr">
+      <c r="AB2" s="6" t="inlineStr">
         <is>
           <t>medication_name</t>
         </is>
       </c>
-      <c r="AB2" s="6" t="inlineStr">
+      <c r="AC2" s="6" t="inlineStr">
         <is>
           <t>medication_dosage</t>
         </is>
       </c>
-      <c r="AC2" s="6" t="inlineStr">
+      <c r="AD2" s="6" t="inlineStr">
         <is>
           <t>medication_frequency</t>
         </is>
       </c>
-      <c r="AD2" s="6" t="inlineStr">
+      <c r="AE2" s="6" t="inlineStr">
         <is>
           <t>medication_duration_days</t>
         </is>
       </c>
-      <c r="AE2" s="6" t="inlineStr">
+      <c r="AF2" s="6" t="inlineStr">
         <is>
           <t>lab_test_name</t>
         </is>
       </c>
-      <c r="AF2" s="6" t="inlineStr">
+      <c r="AG2" s="6" t="inlineStr">
         <is>
           <t>lab_test_loinc_code</t>
         </is>
       </c>
-      <c r="AG2" s="6" t="inlineStr">
+      <c r="AH2" s="6" t="inlineStr">
         <is>
           <t>lab_result_value</t>
         </is>
       </c>
-      <c r="AH2" s="6" t="inlineStr">
+      <c r="AI2" s="6" t="inlineStr">
         <is>
           <t>allergy_text</t>
         </is>
       </c>
-      <c r="AI2" s="6" t="inlineStr">
+      <c r="AJ2" s="6" t="inlineStr">
         <is>
           <t>allergy_category</t>
         </is>
       </c>
-      <c r="AJ2" s="6" t="inlineStr">
+      <c r="AK2" s="6" t="inlineStr">
         <is>
           <t>advice_notes</t>
         </is>
       </c>
-      <c r="AK2" s="6" t="inlineStr">
+      <c r="AL2" s="6" t="inlineStr">
         <is>
           <t>clinical_notes</t>
         </is>
       </c>
-      <c r="AL2" s="6" t="inlineStr">
+      <c r="AM2" s="6" t="inlineStr">
         <is>
           <t>follow_up_date</t>
         </is>
       </c>
-      <c r="AM2" s="6" t="inlineStr">
+      <c r="AN2" s="6" t="inlineStr">
         <is>
           <t>family_history_text</t>
         </is>
       </c>
-      <c r="AN2" s="6" t="inlineStr">
+      <c r="AO2" s="6" t="inlineStr">
         <is>
           <t>document_type</t>
         </is>
       </c>
-      <c r="AO2" s="6" t="inlineStr">
+      <c r="AP2" s="6" t="inlineStr">
         <is>
           <t>document_filename</t>
         </is>
       </c>
-      <c r="AP2" s="6" t="inlineStr">
+      <c r="AQ2" s="6" t="inlineStr">
         <is>
           <t>immunization_vaccine_name</t>
         </is>
       </c>
-      <c r="AQ2" s="6" t="inlineStr">
+      <c r="AR2" s="7" t="inlineStr">
         <is>
           <t>immunization_date</t>
         </is>
       </c>
-      <c r="AR2" s="7" t="inlineStr">
+      <c r="AS2" s="7" t="inlineStr">
         <is>
           <t>hi_type</t>
         </is>
       </c>
-      <c r="AS2" s="7" t="inlineStr">
+      <c r="AT2" s="7" t="inlineStr">
         <is>
           <t>hi_types_multi</t>
         </is>
       </c>
-      <c r="AT2" s="7" t="inlineStr">
+      <c r="AU2" s="7" t="inlineStr">
         <is>
           <t>care_context_id</t>
         </is>
       </c>
-      <c r="AU2" s="7" t="inlineStr">
+      <c r="AV2" s="7" t="inlineStr">
         <is>
           <t>display</t>
         </is>
       </c>
-      <c r="AV2" s="7" t="inlineStr">
+      <c r="AW2" s="7" t="inlineStr">
         <is>
           <t>link_request_status</t>
         </is>
       </c>
-      <c r="AW2" s="7" t="inlineStr">
+      <c r="AX2" s="7" t="inlineStr">
         <is>
           <t>link_status</t>
         </is>
       </c>
-      <c r="AX2" s="7" t="inlineStr">
+      <c r="AY2" s="7" t="inlineStr">
         <is>
           <t>link_error</t>
         </is>
       </c>
-      <c r="AY2" s="7" t="inlineStr">
+      <c r="AZ2" s="8" t="inlineStr">
         <is>
           <t>linked_at</t>
         </is>
       </c>
-      <c r="AZ2" s="8" t="inlineStr">
+      <c r="BA2" s="8" t="inlineStr">
         <is>
           <t>consent_status</t>
         </is>
       </c>
-      <c r="BA2" s="8" t="inlineStr">
+      <c r="BB2" s="8" t="inlineStr">
         <is>
           <t>consent_artifact_id</t>
         </is>
       </c>
-      <c r="BB2" s="8" t="inlineStr">
+      <c r="BC2" s="8" t="inlineStr">
         <is>
           <t>hiu_id</t>
         </is>
       </c>
-      <c r="BC2" s="8" t="inlineStr">
+      <c r="BD2" s="8" t="inlineStr">
         <is>
           <t>bundle_created_at</t>
         </is>
       </c>
-      <c r="BD2" s="8" t="inlineStr">
+      <c r="BE2" s="8" t="inlineStr">
         <is>
           <t>bundle_transfer_status</t>
         </is>
       </c>
-      <c r="BE2" s="8" t="inlineStr">
+      <c r="BF2" s="8" t="inlineStr">
         <is>
           <t>transfer_error</t>
         </is>
@@ -861,8 +867,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="AR1:AY1"/>
-    <mergeCell ref="AZ1:BE1"/>
     <mergeCell ref="I1:AQ1"/>
+    <mergeCell ref="AZ1:BF1"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>